<commit_message>
Added Rocket CEA Thrust Curve estimation
</commit_message>
<xml_diff>
--- a/RegenSolver/enginefiles/engineparameters.xlsx
+++ b/RegenSolver/enginefiles/engineparameters.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2347036970157674</v>
+        <v>0.2318368170157674</v>
       </c>
     </row>
     <row r="10">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.164380147000313</v>
+        <v>0.161513267000313</v>
       </c>
     </row>
     <row r="14">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.003350371164685926</v>
+        <v>0.001675185582342963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added CEA plot and made some changes to the engine sizing scripts
</commit_message>
<xml_diff>
--- a/RegenSolver/enginefiles/engineparameters.xlsx
+++ b/RegenSolver/enginefiles/engineparameters.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2347036970157674</v>
+        <v>0.2318368170157674</v>
       </c>
     </row>
     <row r="10">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.164380147000313</v>
+        <v>0.161513267000313</v>
       </c>
     </row>
     <row r="14">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.003350371164685926</v>
+        <v>0.001675185582342963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>